<commit_message>
add table of understand 20 reports about web3 Security
</commit_message>
<xml_diff>
--- a/Report20Rs.xlsx
+++ b/Report20Rs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KLTN_Research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98510463-3EB6-40E7-92B7-252DDB76E8B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06A0551-21EE-4AE2-8884-D81A07ADD888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{0D0DBE38-4444-45F0-9753-6DFF1AB9C488}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="158">
   <si>
     <t>Phân Loại Phương Pháp</t>
   </si>
@@ -135,20 +135,6 @@
 (Probabilistic pattern inference).</t>
   </si>
   <si>
-    <t>Trace2Inv (FSE 2024)</t>
-  </si>
-  <si>
-    <t>Khó khăn trong việc khai phá và 
-đánh giá tính hiệu quả 
-thực tế của các bất biến 
-bảo vệ hợp đồng trong thời gian chạy.</t>
-  </si>
-  <si>
-    <t>Phân tích dấu vết giao dịch lịch sử, 
-Khai phá bất biến động, 
-Mô phỏng tấn công.</t>
-  </si>
-  <si>
     <t>LENT-SSE (ISSTA 2024)</t>
   </si>
   <si>
@@ -162,30 +148,7 @@
 Thuật toán thu hồi/bỏ qua đường dẫn.</t>
   </si>
   <si>
-    <t>Midas (ISSTA 2024)</t>
-  </si>
-  <si>
-    <t>Khó khăn trong việc định hướng Fuzzer 
-để khám phá các chuỗi tấn công 
-mang lại lợi nhuận thực tế (Profitable exploits).</t>
-  </si>
-  <si>
-    <t>Fuzzing theo phản hồi lợi nhuận tài chính, 
-Phân tích vi phân (Differential Analysis), 
-Điểm đo lường Waypoint.</t>
-  </si>
-  <si>
     <t>DeFort (ISSTA 2024)</t>
-  </si>
-  <si>
-    <t>Thao túng giá (Price manipulation) 
-đòi hỏi phân tích chuỗi giao dịch phức tạp
-mà các công cụ tĩnh thường bỏ lỡ.</t>
-  </si>
-  <si>
-    <t>Mô hình hóa hành vi bất thường, 
-Giám sát chuỗi (On-chain monitoring), 
-Tính toán lợi nhuận.</t>
   </si>
   <si>
     <t>Nyx (S&amp;P 2024)</t>
@@ -215,19 +178,6 @@
 Bounded Model Checking.</t>
   </si>
   <si>
-    <t>Mau (GPU Fuzzing) (S&amp;P 2024)</t>
-  </si>
-  <si>
-    <t>Thông lượng (throughput) của Fuzzer 
-bị nghẽn do độ trễ của cơ chế 
-đồng thuận và kiến trúc xử lý tuần tự của CPU.</t>
-  </si>
-  <si>
-    <t>Fuzzing tăng tốc bằng GPU, 
-Kiến trúc SIMD, Bộ nhớ lưu trữ tăng dần, 
-Bitmap lưu trạng thái giao dịch.</t>
-  </si>
-  <si>
     <t>Clear (ICSE 2024)</t>
   </si>
   <si>
@@ -269,20 +219,6 @@
 (Graph Attention Network).</t>
   </si>
   <si>
-    <t>ItyFuzz (ISSTA 2023)</t>
-  </si>
-  <si>
-    <t>Khó khăn trong việc mô phỏng, lưu trữ 
-và biến đổi các chuỗi giao dịch dài 
-có trạng thái (stateful) trên blockchain.</t>
-  </si>
-  <si>
-    <t>Fuzzing dựa trên ảnh chụp nhanh 
-(Snapshot-based fuzzer), 
-Cơ chế waypoint luồng dữ liệu, 
-Lưu trữ trạng thái EVM.</t>
-  </si>
-  <si>
     <t>DeFiTainter (ISSTA 2023)</t>
   </si>
   <si>
@@ -309,19 +245,6 @@
 từ phản hồi của bộ xác minh.</t>
   </si>
   <si>
-    <t>TransRacer (FSE 2023)</t>
-  </si>
-  <si>
-    <t>Lỗi tương tranh giao dịch (Transaction race) 
-tiềm ẩn sâu trong các trạng thái hợp đồng 
-cụ thể khó tiếp cận bằng kỹ thuật ngẫu nhiên.</t>
-  </si>
-  <si>
-    <t>Khám phá không gian bằng thực thi ký hiệu, 
-Định hướng tìm kiếm 
-bằng phụ thuộc hàm (Function dependence).</t>
-  </si>
-  <si>
     <t>STT</t>
   </si>
   <si>
@@ -355,13 +278,386 @@
     <t>Chi phi thanh toán và kiểm soát tài nguyên lớn (Cần GPU mạnh);
 Phụ thuộc vào độ chất lượng dữ liệu (DPO); 
 Phạm vi còn chưa nhiểu (4 lỗi chính)</t>
+  </si>
+  <si>
+    <t>CFT --&gt; SFT --&gt; DPO
+-cft = RAG + rule based + LLM
+-sft = CoT layer prompt
+-dpo= multi agentic critique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dùng lại; 
+có thể triển khai theo hướng khác nhưng vấn giữ được tinh thần cốt lõi cua bài báo  </t>
+  </si>
+  <si>
+    <t>Kết quả</t>
+  </si>
+  <si>
+    <t>một hệ thống: ứng dụng một dạng Graph kết hợp với phân tích trước và deep learning thêm thuật toán để gom các anti-reentrency pattern; sự kết hợp này bổ sung cho thiếu sót cho các static tool analysis thông thường nhưu slither/mythril</t>
+  </si>
+  <si>
+    <t>Một hệ thống được nghiên cứu và phát triển để so sánh, đánh giá các SAST thông qua benchmark lớn và taxonomy (hệ thống phân loại lỗ hổng) hiện đại</t>
+  </si>
+  <si>
+    <t>Input: các contract với độ bao phu 40/45 lỗ hổng
+Execution engine: 8 tools chạy trong môi trường cô lập;
+Sau đó, mapping và maching về một chung chuẩn taxonomy 45 loại để đối chiếu
+Analysis module: tính toán, thống kế các hiệu suất đầu ra; mô phỏng chạy nhiều công cụ xem có mang kết quả tốt hơn không</t>
+  </si>
+  <si>
+    <t>3 stage chính:
+1: Data filteration: chọn data dựa trên nguyên tắc:  Ethereum contracts prone to reentrancy attacks are often enforced with anti-reentrancy patterns
+2: RentPDG: retains the structure directly related to anti-reentrency patterns; nodes and edges associated with external call
+3: Model Recognition</t>
+  </si>
+  <si>
+    <t>Một static analysis framework được thiết kế để phát hiện các CCVs ở mức Bytecode; Nhận diện gap của CC: access control completeness &amp; cross-bridge semantic consistency</t>
+  </si>
+  <si>
+    <t>Tính chuyên biệt hóa cao (Đi thẳng vào khoảng trống của web3);
+Giảm thiểu FP khi sử dụng Fine-Grained Analysis - phân tích tĩnh ở level chi tiết;
+Đạt tốc độ cao và tốn ít tài nguyên hơn Fuzzing (cần mô phỏng môi trường)</t>
+  </si>
+  <si>
+    <t>Hạn chế của Static Analysis: Path Explosion: bùng nổ đường dẫn;
+Bỏ qua rủi ro Off-chain: nếu bị đánh cắp key ở đây thì tool vô dụng</t>
+  </si>
+  <si>
+    <t>Bộ phân tích cú pháp: Đọc bytecode chuyển về dạng  IR hoặc AST
+Cross-chain Semantic Extractor: dựa trên IR, gắn label các thành phần đặc thù;
+Fine-Grained Analysis Engine: chạy thuật toán tạo path;
+Vulnerability Detectors: sử dụng các rule được define sẵn và gán lỗi
+Report</t>
+  </si>
+  <si>
+    <t>Precision: 84.95%
+Recall Coverage: 89.77%
+Thử nghiệm trên quy mô lớn: 129 Bridge, 1703 contracts</t>
+  </si>
+  <si>
+    <t>Một hệ thống áp dụng 2 pp; sử dụng Txs đã thực thi và cả những Tx sắp được thực thi tròn Mempool Monitor để mô phỏng được State tree và từ đây áp dụng Symbolic Execution để tạo ra tc và dùng Vulnerability Detector để xác nhận, prune path và đồng thời giảm false positive</t>
+  </si>
+  <si>
+    <t>Giải quyết bottleneck: Path explosion;
+Giảm time;
+Phát hiện được deep-bug và giảm false positive
+Có khả năng phát hiện lỗi trong bối cảnh Miner Extractable Value và các cuộc tấn công hẹp vì phân tích trên mempool</t>
+  </si>
+  <si>
+    <t>Tính thực tế cao (SA được tiến gần với live blockchain);
+Chủ động phát hiện lỗi (Near TXs);
+Giải quyết được vấn đề Scalability của Symbolic Execution</t>
+  </si>
+  <si>
+    <t>Phụ thuộc vào State Bias: phát hiện lỗi tốt xung quanh 
+state hiện tại, tuy nhiên khả năng không phát hiện bug đối với các 
+TXs đặc biệt hoặc chưa chạm tới trong MEMPOOL; 
+thách thức kỹ thuật khi liên tục giám sát MEMPool, giả lập trạng thái</t>
+  </si>
+  <si>
+    <t>Demystifying Invariant Effectiveness for Securing Smart Contracts (FSE 2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not your type! Detecting storage collision vulnerabilities... (NDSS 2024) </t>
+  </si>
+  <si>
+    <t>Advanced smart contract vulnerability detection via LLM-powered multi-agent systems (TSE 2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vulseye: Detect Smart Contract Vulnerabilities via Stateful Directed... (TIFS 2025) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">When ChatGPT Meets Smart Contract Vulnerability Detection... (TOSEM 2025) </t>
+  </si>
+  <si>
+    <t>Đạt hiệu suất vượt trội, cung cấp khả năng giải thích nguyên nhân gốc rễ rõ ràng, phát hiện được các lỗi phức tạp.</t>
+  </si>
+  <si>
+    <t>Đề xuất khung kiểm thử phân biệt kết hợp LLM để tự động sinh các hợp đồng seed và phát hiện sự không nhất quán giữa các máy ảo EVM.</t>
+  </si>
+  <si>
+    <t>Tìm ra 26 lỗi chưa từng được biết đến trên 9 EVM (22 lỗi được xác nhận), tăng độ bao phủ mã lên tới 65%.</t>
+  </si>
+  <si>
+    <t>Khám phá các lỗi cốt lõi ở tầng kiến trúc ảo (EVM) 
+thay vì chỉ dừng ở tầng hợp đồng, 
+giải quyết tốt các lỗi từ chối dịch vụ (DoS).</t>
+  </si>
+  <si>
+    <t>Đòi hỏi chi phí và tài nguyên 
+thiết lập phức tạp (nhiều môi trường EVM) để đối chiếu, phụ thuộc vào 
+hiệu suất của LLM để tìm nguyên nhân gốc.</t>
+  </si>
+  <si>
+    <t>Nhận diện thành công 12 mẫu chống tái xâm nhập phổ biến (trong đó có 8 mẫu hoàn toàn mới), giúp giảm hơn 85% tỷ lệ cảnh báo sai (FPs) khi tích hợp vào các công cụ phân tích hiện có.</t>
+  </si>
+  <si>
+    <t>Khắc phục được nhược điểm chí mạng của các công cụ quét tĩnh (báo lỗi sai quá nhiều), tự động học các mẫu bảo vệ phức tạp mà không cần chuyên gia định nghĩa thủ công.</t>
+  </si>
+  <si>
+    <t>Chỉ tập trung vào việc lọc cảnh báo sai cho một loại lỗi duy nhất (Reentrancy), không mang tính đa dụng để trực tiếp tìm ra các loại lỗ hổng bảo mật mới.</t>
+  </si>
+  <si>
+    <t>Tự động sinh ra các thuộc tính kiểm chứng cho hợp đồng bằng cách kết hợp LLM và RAG, sau đó đưa vào Prover để kiểm chứng hình thức.</t>
+  </si>
+  <si>
+    <t>Đạt độ bao phủ 80% so với nhãn gốc, phát hiện 26 CVEs thực tế và 12 lỗ hổng zero-day (nhận được bug bounty).</t>
+  </si>
+  <si>
+    <t>Tự động hóa được khâu tốn công sức và khó nhất 
+của Formal Verification là "định nghĩa thuộc tính", tính bao quát cao.</t>
+  </si>
+  <si>
+    <t>Kết quả đầu ra bị giới hạn bởi chất lượng 
+dữ liệu nền tảng RAG; có thể bỏ sót các thuộc
+ tính nghiệp vụ quá dị biệt hoặc chưa từng có tiền lệ.</t>
+  </si>
+  <si>
+    <t>Đánh giá trên 10.394 lỗ hổng cho thấy các công cụ SAST hiện tại bỏ sót tới 50% lỗi, độ chính xác (precision) chưa tới 10%, và cực kỳ yếu ở các lỗi logic nằm ngoài Access Control và Reentrancy.</t>
+  </si>
+  <si>
+    <t>Cung cấp một bộ dữ liệu tiêu chuẩn cực kỳ đồ sộ, đa dạng và cập nhật, tạo nền tảng vững chắc và hệ quy chiếu chuẩn xác để đo lường các công cụ trong tương lai.</t>
+  </si>
+  <si>
+    <t>Bản chất đây là một bài báo nghiên cứu đánh giá (Empirical Study), không đề xuất một công cụ, mô hình hay thuật toán mới để trực tiếp khắc phục các điểm yếu của phân tích tĩnh.</t>
+  </si>
+  <si>
+    <t>Fuzzing truyền thống khó tạo ra chuỗi giao dịch 
+để chạm tới các lỗi nằm sâu bên trong 
+các nhánh hợp đồng phức tạp.</t>
+  </si>
+  <si>
+    <t>Đề xuất một fuzzer có hướng (Directed Fuzzing) nhận thức được trạng thái, hướng dẫn tự động tạo chuỗi giao dịch đi sâu vào đồ thị luồng dữ liệu.</t>
+  </si>
+  <si>
+    <t>Fuzzing có hướng (Stateful Directed Fuzzing), Phân tích Đồ thị luồng điều khiển/dữ liệu, Sinh chuỗi trạng thái (State Sequence Generation).</t>
+  </si>
+  <si>
+    <t>Kích hoạt hiệu quả các trạng thái lỗi ẩn sâu mà các công cụ Fuzzing truyền thống không thể chạm tới.</t>
+  </si>
+  <si>
+    <t>Giảm thiểu việc thử nghiệm 
+ngẫu nhiên vô ích, tối ưu hóa thời gian 
+và năng lực tính toán để nhắm thẳng vào các mục tiêu nghi ngờ.</t>
+  </si>
+  <si>
+    <t>Cần phải có một bước phân tích 
+tĩnh đủ tốt để khoanh vùng mục tiêu trước, 
+nếu khoanh vùng sai sẽ làm giảm hiệu suất.</t>
+  </si>
+  <si>
+    <t>Thiếu đánh giá thực tế về mức độ hiệu quả của việc triển khai các cơ chế bảo vệ "bất biến" (invariants) chặn giao dịch trên mạng lưới.</t>
+  </si>
+  <si>
+    <t>Dùng công cụ Trace2Inv để tự động trích xuất các quy tắc bất biến từ lịch sử giao dịch và đánh giá tính thực tiễn của 23 mẫu bất biến phổ biến.</t>
+  </si>
+  <si>
+    <t>Phân tích dấu vết và luồng truyền bẩn (Trace &amp; dynamic taint analysis), Invariant Synthesis (Trace2Inv).</t>
+  </si>
+  <si>
+    <t>Các bất biến kết hợp chặn thành công &gt;74% đến 85% các cuộc tấn công exploit, với tỷ lệ dương tính giả cực thấp (chỉ ~0.3%).</t>
+  </si>
+  <si>
+    <t>Cho cái nhìn định lượng cực kỳ giá trị, 
+bất biến có thể chặn tấn công trực tiếp on-chain 
+theo thời gian thực rất hữu hiệu.</t>
+  </si>
+  <si>
+    <t>Kẻ tấn công hoặc người dùng tinh vi có thể 
+chia nhỏ giao dịch để lách qua (bypass) bộ chặn bất biến, gây khó chịu cho người dùng thông thường.</t>
+  </si>
+  <si>
+    <t>Thao túng giá (Price manipulation) 
+đòi hỏi phân tích chuỗi giao dịch phức tạp
+mà các công cụ tĩnh thường bỏ lỡ / Các công cụ hiện tại phản ứng chậm hoặc quá cứng nhắc trước các lỗ hổng thao túng giá tài chính (như Flash loans) trong DeFi.</t>
+  </si>
+  <si>
+    <t>Khung giám sát tự động phân tích hành vi thao túng giá DeFi bằng cách theo dõi sự biến động của tỷ giá token kết hợp với phân tích hành vi sinh lời.</t>
+  </si>
+  <si>
+    <t>Mô hình hóa hành vi bất thường, 
+Giám sát chuỗi (On-chain monitoring), 
+Tính toán lợi nhuận / Mô hình hành vi thao túng giá (Behavior models), Chiến lược giám sát biến động giá, Phân tích lợi nhuận động (Dynamic profit tracking).</t>
+  </si>
+  <si>
+    <t>Vượt trội so với các hệ thống phân tích giá khác, tự động định vị chính xác giao dịch, kẻ tấn công và nạn nhân.</t>
+  </si>
+  <si>
+    <t>Nhạy bén cao với các lỗ hổng 
+mang nặng tính logic kinh tế/tài chính (DeFi semantics) - điểm mù của 
+phân tích mã nguồn đơn thuần.</t>
+  </si>
+  <si>
+    <t>Phạm vi hẹp, chủ yếu xoay quanh 
+hệ sinh thái DEX/Pool giá, khó phát 
+hiện các vụ hack chiếm đoạt qua kiểm soát quyền (Access Control).</t>
+  </si>
+  <si>
+    <t>Dùng chiến lược hai giai đoạn: cắt tỉa tĩnh để loại các cụm mã an toàn, sau đó dùng thực thi biểu tượng để chứng minh lỗi đó có thể trục lợi.</t>
+  </si>
+  <si>
+    <t>Lọc bỏ thành công các báo cáo giả, xác nhận tính khả thi bị khai thác của các lỗ hổng Front-Running với độ chuẩn xác cao.</t>
+  </si>
+  <si>
+    <t>Giảm số lượng lớn báo động giả 
+bằng cách kiểm chứng "điều kiện có lợi nhuận" thay vì 
+chỉ tìm sự phụ thuộc thứ tự giao dịch (TOD).</t>
+  </si>
+  <si>
+    <t>Việc phân tích Symbolic Execution 
+dễ bị bùng nổ đường dẫn (path explosion) khi 
+xử lý các hợp đồng có luồng rẽ nhánh dày đặc.</t>
+  </si>
+  <si>
+    <t>Sử dụng mô hình đa phương thức kết hợp chiến lược prompt ToT để đối chiếu logic giữa mã nguồn và văn bản (tài liệu/comment) để sinh bất biến.</t>
+  </si>
+  <si>
+    <t>Tìm ra 119 lỗi zero-day về logic nghiệp vụ, sinh ra bất biến có độ chính xác rất cao để hỗ trợ công cụ kiểm chứng.</t>
+  </si>
+  <si>
+    <t>Hiểu được "ý định" của nhà phát 
+triển (qua comment/code), xuất sắc trong việc tóm gọn các lỗi logic nghiệp vụ cực khó.</t>
+  </si>
+  <si>
+    <t>Yêu cầu hợp đồng hoặc tập huấn luyện 
+phải có sẵn văn bản mô tả (comments/documentations) đủ tốt để mô hình đa phương thức học hỏi.</t>
+  </si>
+  <si>
+    <t>Các hợp đồng nâng cấp (Upgradeable) qua Proxy thường xuyên gặp lỗi xung đột bố cục lưu trữ (storage collision), gây mất kiểm soát hoặc đè dữ liệu.</t>
+  </si>
+  <si>
+    <t>Quét toàn bộ on-chain Ethereum để phát hiện các hợp đồng bị lệch kiểu lưu trữ do delegatecall, và tự động sinh mã khai thác (exploit) thông qua CRUSH.</t>
+  </si>
+  <si>
+    <t>Phân tích bố cục lưu trữ (Storage Layout Analysis), Trích xuất Bytecode, Tự động tổng hợp mã khai thác (Automated exploit synthesis).</t>
+  </si>
+  <si>
+    <t>Quét &gt;14 triệu hợp đồng, tìm ra gần 15.000 hợp đồng rủi ro, sinh tự động 956 PoC với thiệt hại ước tính tiềm ẩn 6 triệu USD.</t>
+  </si>
+  <si>
+    <t>Khung phân tích đầu tiên và 
+quy mô lớn nhất tính đến nay tập trung giải quyết triệt để lỗi xung đột lưu trữ Proxy.</t>
+  </si>
+  <si>
+    <t>Thu hẹp phạm vi ở các mẫu hợp đồng 
+sử dụng kiến trúc nâng cấp (Proxy Pattern/Delegatecall), không giải quát được lỗi logic khác.</t>
+  </si>
+  <si>
+    <t>Nâng cao khả năng phát hiện bằng cách dùng Học đối chiếu (Contrastive Learning) nhằm khai thác sự tương đồng và khác biệt giữa các nhóm hợp đồng.</t>
+  </si>
+  <si>
+    <t>Cho F1-score cao hơn từ 9.73% đến 39.99% so với 13 công cụ Deep Learning tiên tiến hiện tại.</t>
+  </si>
+  <si>
+    <t>Mô hình có khả năng tổng quát hóa cực tốt, 
+có khả năng phân biệt đặc trưng lỗ hổng kể cả trên mã nguồn bị xáo trộn.</t>
+  </si>
+  <si>
+    <t>Cần một lượng lớn dữ liệu gán nhãn tốt để huấn luyện CL; bản chất mô hình là hộp đen nên 
+tính giải thích nguyên nhân lỗi rất thấp.</t>
+  </si>
+  <si>
+    <t>Kết hợp mô hình ngôn ngữ lớn (GPT) với phân tích chương trình tĩnh để phát hiện các lỗ hổng logic nghiệp vụ khó tìm.</t>
+  </si>
+  <si>
+    <t>Đạt độ chính xác cao trong việc phát hiện lỗ hổng logic, giảm đáng kể tỷ lệ dương tính giả (false positives).</t>
+  </si>
+  <si>
+    <t>Nắm bắt được ý định của nhà phát triển, 
+xử lý tốt logic nghiệp vụ và ngữ cảnh của code.</t>
+  </si>
+  <si>
+    <t>Tốn chi phí gọi API và thời gian xử lý 
+chậm hơn các luồng phân tích tĩnh thuần túy.</t>
+  </si>
+  <si>
+    <t>Học và trích xuất đặc trưng ngữ nghĩa từ mã nguồn để tự động nhận diện lỗ hổng mà không cần định nghĩa quy tắc thủ công.</t>
+  </si>
+  <si>
+    <t>Cải thiện đáng kể hiệu suất so với các phương pháp học sâu và phân tích tĩnh truyền thống nhờ nhận diện tốt cấu trúc đồ thị.</t>
+  </si>
+  <si>
+    <t>Khả năng tự động học trích xuất đặc trưng 
+cực tốt, linh hoạt cao với nhiều mẫu mã nguồn mới.</t>
+  </si>
+  <si>
+    <t>Yêu cầu tài nguyên huấn luyện lớn, kết quả của mô 
+hình mang tính "hộp đen" và khó giải thích nguyên nhân gốc rễ.</t>
+  </si>
+  <si>
+    <t>Thiếu công cụ kiểm toán tự động có thể bao quát toàn diện các loại lỗ hổng phức tạp với độ chính xác cao.</t>
+  </si>
+  <si>
+    <t>Đề xuất khung LLM-SmartAudit sử dụng hệ thống hội thoại đa tác tử lặp lại để đánh giá và tìm kiếm lỗ hổng trong hợp đồng.</t>
+  </si>
+  <si>
+    <t>Kiến trúc hội thoại đa tác tử (Multi-agent architecture), Cơ chế Buffer-of-thought, LLMs.</t>
+  </si>
+  <si>
+    <t>Đạt 98% độ chính xác trên các lỗ hổng phổ biến, phát hiện 12/13 lỗi CVE thực tế, vượt trội hơn các công cụ khác.</t>
+  </si>
+  <si>
+    <t>Tận dụng sự cộng tác của nhiều agent 
+chuyên biệt để phân tích sâu rộng toàn bộ các lỗi khác nhau.</t>
+  </si>
+  <si>
+    <t>Mang nặng tính chất sản phẩm đóng, 
+thiết kế agentic cồng kềnh và thiếu không gian nếu muốn nghiên cứu tối ưu hóa tài nguyên trực tiếp tại tầng kiến trúc hệ thống cốt lõi.</t>
+  </si>
+  <si>
+    <t>Tập trung theo dõi và phát hiện các đường dẫn luồng dữ liệu thao túng giá xuyên suốt các giao thức DeFi.</t>
+  </si>
+  <si>
+    <t>Lập bản đồ thành công và phát hiện chính xác nhiều lỗ hổng thao túng giá thực tế trên các dự án.</t>
+  </si>
+  <si>
+    <t>Mô hình hóa chính xác các lời gọi hàm đan chéo phức tạp, 
+đặc biệt hiệu quả với tấn công liên quan đến Oracle/Flashloan.</t>
+  </si>
+  <si>
+    <t>Có thể xảy ra hiện tượng over-approximation
+ dẫn đến báo lỗi giả ở các giao thức quá phức tạp.</t>
+  </si>
+  <si>
+    <t>Tự động hóa quá trình sinh và xác minh bản vá lỗi cho hợp đồng thông minh bằng cách tăng tốc qua mô hình thống kê.</t>
+  </si>
+  <si>
+    <t>Vá tự động và song song hàng loạt hợp đồng có lỗ hổng bảo mật với tỷ lệ sinh bản vá chuẩn xác cao.</t>
+  </si>
+  <si>
+    <t>Tiết kiệm tối đa thời gian vá lỗi, tăng tốc độ kiểm tra 
+tính đúng đắn của bản vá so với các phương pháp cũ.</t>
+  </si>
+  <si>
+    <t>Không hoàn toàn đảm bảo việc tối ưu hóa lượng phí 
+Gas sau khi sửa lỗi, chỉ giới hạn hiệu quả ở những lỗi mà mô hình đã học trước đó.</t>
+  </si>
+  <si>
+    <t>Cần xác định năng lực và giới hạn thực tế của các LLM (như ChatGPT) trong bảo mật hợp đồng thông minh so với các phương pháp cũ.</t>
+  </si>
+  <si>
+    <t>Một báo cáo nghiên cứu đánh giá toàn diện năng lực của LLM qua kỹ thuật Prompting, đồng thời đề xuất cách dùng RAG để rà soát "bad practices".</t>
+  </si>
+  <si>
+    <t>Đánh giá LLM thực nghiệm, RAG, Kỹ thuật Prompt lùi bước (Step-Back Prompting).</t>
+  </si>
+  <si>
+    <t>LLM phát hiện rất tốt các thực tiễn lập trình kém (bad practices) và lỗ hổng mức ngữ nghĩa, nhưng còn yếu ở các cấu trúc thực thi dài hạn.</t>
+  </si>
+  <si>
+    <t>Mang đến một cái nhìn định lượng, 
+khách quan và đưa ra hướng dẫn rõ ràng (ví dụ: dùng Step-Back Prompting) để tối đa sức mạnh của LLM.</t>
+  </si>
+  <si>
+    <t>Đây là bài báo thiên về phân tích và 
+đánh giá mô hình sẵn có (ChatGPT) thay vì đề xuất một mô hình/thuật toán phát hiện lỗ hổng chuyên biệt mới.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -392,8 +688,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -409,6 +720,18 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -451,12 +774,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -465,14 +789,39 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="60% - Accent1" xfId="2" builtinId="32"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
@@ -786,24 +1135,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8506608-C8FB-4540-85FD-03E2E1E50776}">
-  <dimension ref="A3:H23"/>
+  <dimension ref="A3:L23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
     <col min="2" max="2" width="36.85546875" customWidth="1"/>
     <col min="3" max="3" width="37" customWidth="1"/>
     <col min="4" max="5" width="45.140625" customWidth="1"/>
-    <col min="6" max="6" width="45.28515625" customWidth="1"/>
-    <col min="7" max="7" width="30" customWidth="1"/>
-    <col min="8" max="8" width="33.28515625" customWidth="1"/>
+    <col min="6" max="7" width="45.28515625" customWidth="1"/>
+    <col min="8" max="8" width="40.7109375" customWidth="1"/>
+    <col min="9" max="9" width="50.7109375" customWidth="1"/>
+    <col min="11" max="11" width="45.140625" customWidth="1"/>
+    <col min="12" max="12" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>0</v>
@@ -812,46 +1163,58 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="102.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+        <v>50</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="102.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="C4" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+      <c r="E4" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -863,35 +1226,59 @@
       <c r="D5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="2"/>
+      <c r="E5" s="2" t="s">
+        <v>80</v>
+      </c>
       <c r="F5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-    </row>
-    <row r="6" spans="1:8" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="G5" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+    </row>
+    <row r="6" spans="1:12" ht="108.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
         <v>3</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2" t="s">
+      <c r="E6" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-    </row>
-    <row r="7" spans="1:8" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="G6" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="L6" s="7"/>
+    </row>
+    <row r="7" spans="1:12" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -903,332 +1290,523 @@
       <c r="D7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="2"/>
+      <c r="E7" s="2" t="s">
+        <v>87</v>
+      </c>
       <c r="F7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-    </row>
-    <row r="8" spans="1:8" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+      <c r="G7" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+    </row>
+    <row r="8" spans="1:12" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
         <v>5</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2" t="s">
+      <c r="E8" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-    </row>
-    <row r="9" spans="1:8" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+      <c r="G8" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="L8" s="7"/>
+    </row>
+    <row r="9" spans="1:12" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6">
         <v>6</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2" t="s">
+      <c r="E9" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-    </row>
-    <row r="10" spans="1:8" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+      <c r="G9" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="L9" s="7"/>
+    </row>
+    <row r="10" spans="1:12" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="12">
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+    </row>
+    <row r="11" spans="1:12" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="9">
+        <v>8</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2" t="s">
+      <c r="E11" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-    </row>
-    <row r="11" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
-        <v>8</v>
-      </c>
-      <c r="B11" s="2" t="s">
+      <c r="G11" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+    </row>
+    <row r="12" spans="1:12" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6">
+        <v>9</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+    </row>
+    <row r="13" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="12">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-    </row>
-    <row r="12" spans="1:8" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
-        <v>9</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
-        <v>10</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="2"/>
+        <v>106</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>107</v>
+      </c>
       <c r="F13" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-    </row>
-    <row r="14" spans="1:8" ht="90.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+        <v>108</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+    </row>
+    <row r="14" spans="1:12" ht="90.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="12">
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E14" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="F14" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-    </row>
-    <row r="15" spans="1:8" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+        <v>29</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+    </row>
+    <row r="15" spans="1:12" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="12">
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>116</v>
+      </c>
       <c r="F15" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-    </row>
-    <row r="16" spans="1:8" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+        <v>32</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+    </row>
+    <row r="16" spans="1:12" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="6">
         <v>13</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-    </row>
-    <row r="17" spans="1:8" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+      <c r="B16" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+    </row>
+    <row r="17" spans="1:12" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6">
         <v>14</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="B17" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-    </row>
-    <row r="18" spans="1:8" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+      <c r="D17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+    </row>
+    <row r="18" spans="1:12" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="12">
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E18" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>130</v>
+      </c>
       <c r="F18" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-    </row>
-    <row r="19" spans="1:8" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+        <v>38</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+    </row>
+    <row r="19" spans="1:12" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="6">
         <v>16</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="B19" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-    </row>
-    <row r="20" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+      <c r="D19" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+    </row>
+    <row r="20" spans="1:12" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="12">
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20" s="2"/>
+        <v>138</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>139</v>
+      </c>
       <c r="F20" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-    </row>
-    <row r="21" spans="1:8" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+        <v>140</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="K20" s="7"/>
+      <c r="L20" s="7"/>
+    </row>
+    <row r="21" spans="1:12" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6">
         <v>18</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C21" s="2" t="s">
+      <c r="B21" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-    </row>
-    <row r="22" spans="1:8" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+      <c r="D21" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="K21" s="7"/>
+      <c r="L21" s="7"/>
+    </row>
+    <row r="22" spans="1:12" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="12">
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E22" s="2"/>
+        <v>46</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>148</v>
+      </c>
       <c r="F22" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-    </row>
-    <row r="23" spans="1:8" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+        <v>47</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+    </row>
+    <row r="23" spans="1:12" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="12">
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E23" s="2"/>
+        <v>152</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>153</v>
+      </c>
       <c r="F23" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
+        <v>154</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>